<commit_message>
Atualiza base de clientes: novos grupos e status de implantação
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/base/base implantação.xlsx
+++ b/data/base/base implantação.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgcontecnica1-my.sharepoint.com/personal/warruda_mgcontecnica_com_br/Documents/Documentos/python/Portal-implantacao-tmp/data/base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3D9C078-0120-44A4-A4DA-261C6F599853}"/>
+  <xr:revisionPtr revIDLastSave="279" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6CD88D2-17A5-4C6C-8E30-82310FFEC7E1}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-1260" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="221">
   <si>
     <t>ID</t>
   </si>
@@ -479,29 +479,245 @@
   </si>
   <si>
     <t>lagoa-bonita</t>
+  </si>
+  <si>
+    <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+  </si>
+  <si>
+    <t>RK</t>
+  </si>
+  <si>
+    <t>Vander Silva;</t>
+  </si>
+  <si>
+    <t>Victoria Virgens;</t>
+  </si>
+  <si>
+    <t>Reynaldo Santos;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R MICHELÂNGELO, Num.: 191 Comple.: , Bairro: JARDIM MITSUTANI / </t>
+  </si>
+  <si>
+    <t>SERGIO@PLASTICOSINDEP.COM.BR;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11) 91648-5026 / </t>
+  </si>
+  <si>
+    <t>GABRIEL PALADINO RAUNAIMER; BRUNO PALADINO RAUNAIMER;</t>
+  </si>
+  <si>
+    <t>RK - INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua Ourinhos, Num.: 205 Comple.: , Bairro: Parque Industrial das Oliveiras / </t>
+  </si>
+  <si>
+    <t>sergio@plasticosindep.com.br;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 91648-5026 / </t>
+  </si>
+  <si>
+    <t>SERGIO TADEU RAUNAIMER;ELAINE APARECIDA MOLINARI ZAMORA;</t>
+  </si>
+  <si>
+    <t>SANTOS &amp; DIAN MATERIAIS PARA CONSTRUCAO LTDA</t>
+  </si>
+  <si>
+    <t>SD MATERIAIS</t>
+  </si>
+  <si>
+    <t>Bruno Contieri;</t>
+  </si>
+  <si>
+    <t>Daniela Silva;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVENIDA PROFESSOR PEDRO CLARISMUNDO FORNARI, Num.: 1490 Comple.: , Bairro: ENGORDADOURO / </t>
+  </si>
+  <si>
+    <t>financeiro@sdmaterialdeconstrucao.com.br;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11) 4582-5121 / </t>
+  </si>
+  <si>
+    <t>WILSON APARECIDO DIAN;</t>
+  </si>
+  <si>
+    <t>COMERCIO VAREJISTA DE MERCADORIAS 3M LTDA (MATRIZ)</t>
+  </si>
+  <si>
+    <t>SUPERMERCADO 3M</t>
+  </si>
+  <si>
+    <t>Daniel Oliveira;</t>
+  </si>
+  <si>
+    <t>Clara Maria;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua Alberto Borges Soveral, Num.: 09 Comple.: COM FUNDOS PARA A RUA PIETRO DA MILANO 55, Bairro: Parque Independência / </t>
+  </si>
+  <si>
+    <t>MARCOSMARTINS@SUPERMERCADO3M.COM.BR;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 5832-2100 Ramal 229 - Cel: 11 95911-9371 / </t>
+  </si>
+  <si>
+    <t>AA&amp;amp;MARTINS PARTICIPACOES LTDA;ADRIANO AUGUSTO MARTINS;E&amp;amp;G MARTINS PARTICIPACOES LTDA;EDUARDO DE JESUS MARTINS; B&amp;amp;SOLAR PARTICIPACOES LTDA;MARCOS MARQUES MARTINS;</t>
+  </si>
+  <si>
+    <t>COMERCIO VAREJISTA DE MERCADORIAS 3M LTDA (FILIAL 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua Feitiço da Vila, Num.: 36 Comple.: , Bairro: Chácara Santa Maria / </t>
+  </si>
+  <si>
+    <t>ADRIANO AUGUSTO MARTINS;EDUARDO DE JESUS MARTINS;AA&amp;amp;MARTINS PARTICIPACOES LTDA;MARCOS MARQUES MARTINS; B&amp;amp;SOLAR PARTICIPACOES LTDA;E&amp;amp;G MARTINS PARTICIPACOES LTDA;</t>
+  </si>
+  <si>
+    <t>MARQUES &amp; MARTINS ADMINISTRADORA DE BENS PROPRIOS LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avenida Giovanni Gronchi, Num.: 6195 Comple.: SALA 813, Bairro: Vila Andrade / </t>
+  </si>
+  <si>
+    <t>marcosmartins@supermercado3m.com.br;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11) 5832-2100 / </t>
+  </si>
+  <si>
+    <t>Holding</t>
+  </si>
+  <si>
+    <t>MARCOS MARQUES MARTINS;</t>
+  </si>
+  <si>
+    <t>FRUTAS DA TERRA HORTIFRUTI LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rua Alberto Borges Soveral, Num.: 23 Comple.: , Bairro: Parque Independência / </t>
+  </si>
+  <si>
+    <t>contabil@supermercados3m.com.br;</t>
+  </si>
+  <si>
+    <t>E&amp;G MARTINS PARTICIPAÇÕES LTDA</t>
+  </si>
+  <si>
+    <t>Karine Gusmão;</t>
+  </si>
+  <si>
+    <t>Isabelli Afonso;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avenida Giovanni Gronchi, Num.: 6195 Comple.: Sala 813, Bairro: Vila Andrade / </t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11) 4741-0807 / </t>
+  </si>
+  <si>
+    <t>EDUARDO DE JESUS MARTINS;</t>
+  </si>
+  <si>
+    <t>E&amp;G MARTINS ADMINISTRACAO DE BENS PROPRIOS LTDA</t>
+  </si>
+  <si>
+    <t>B&amp;SOLAR PARTICIPACOES LTDA</t>
+  </si>
+  <si>
+    <t>B&amp;SOLAR ADMINISTRACAO DE BENS PROPRIOS LTDA</t>
+  </si>
+  <si>
+    <t>AA&amp;MARTINS ADMINISTRACAO DE BENS PROPRIOS LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avenida Giovanni Gronchi, Num.: 6195 Comple.: Sala 13, Bairro: Vila Andrade / </t>
+  </si>
+  <si>
+    <t>ADRIANO AUGUSTO MARTINS;</t>
+  </si>
+  <si>
+    <t>AA&amp;MARTINS PARTICIPACOES LTDA</t>
+  </si>
+  <si>
+    <t>ALDENIR VENANCIO DE OLIVEIRA LTDA</t>
+  </si>
+  <si>
+    <t>SUPERMERCADO CRISTO REI</t>
+  </si>
+  <si>
+    <t>Ricardo Ferreira;</t>
+  </si>
+  <si>
+    <t>GOMES SERVIÇOS - LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUA JERÔNIMO VILELA, Num.: 271 Comple.: QUADRA 27 LOTE 13, Bairro: VILA SOFIA / </t>
+  </si>
+  <si>
+    <t>venanciopardal@hotmail.com;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64 996444975 / </t>
+  </si>
+  <si>
+    <t>ALDENIR VENANCIO DE OLIVEIRA;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUA MINAS GERAIS, Num.: 698 Comple.: QUADRA 48 - LOTE 10A - SALA 01, Bairro: VILA SANTA MARIA / </t>
+  </si>
+  <si>
+    <t>alineferasoadm@hotmial.com;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(64) 99647-7060 / </t>
+  </si>
+  <si>
+    <t>ARMANDO GOMES DE ASSIS;</t>
+  </si>
+  <si>
+    <t>E&amp;amp;G MARTINS PARTICIPACOES LTDA;EDUARDO DE JESUS MARTINS; AA&amp;amp;MARTINS PARTICIPACOES LTDA;ADRIANO AUGUSTO MARTINS; B&amp;amp;SOLAR PARTICIPACOES LTDA;MARCOS MARQUES MARTINS;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0E6F5"/>
+        <bgColor rgb="FFC0E6F5"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -518,27 +734,16 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="1">
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -553,20 +758,16 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:T19">
-  <autoFilter ref="A1:T19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:T34">
+  <autoFilter ref="A1:T34" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T19">
-    <sortCondition ref="T1:T19"/>
+    <sortCondition ref="D1:D19"/>
   </sortState>
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" totalsRowFunction="average"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="RazaoSocial" totalsRowFunction="average"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ContratoMG" totalsRowFunction="average" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ContratoMG" totalsRowFunction="average" dataDxfId="0"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Grupo" totalsRowFunction="average"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Gerente" totalsRowFunction="average"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Secretaria" totalsRowFunction="average"/>
@@ -578,14 +779,14 @@
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Segmento" totalsRowFunction="average"/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Socio" totalsRowFunction="average"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Implantação CTB"/>
-    <tableColumn id="7" xr3:uid="{0AFAB906-C921-447F-AE27-262AE6DF88B4}" name="Implantação CTB - Realizada" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{0AFAB906-C921-447F-AE27-262AE6DF88B4}" name="Implantação CTB - Realizada"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Implantação EF"/>
-    <tableColumn id="8" xr3:uid="{5B2D038A-745A-4A1C-8CCD-0A7265A0AA57}" name="Implantação EF - Realizada" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{5B2D038A-745A-4A1C-8CCD-0A7265A0AA57}" name="Implantação EF - Realizada"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Implantação DP"/>
     <tableColumn id="9" xr3:uid="{4EC4A72A-B6C2-47C3-A66B-DB898C2CE30E}" name="Implantação DP - Realizada"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="GrupoID"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -906,12 +1107,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T19"/>
+  <dimension ref="A1:T34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
@@ -938,7 +1139,7 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -1160,6 +1361,9 @@
       <c r="Q4" t="s">
         <v>149</v>
       </c>
+      <c r="R4">
+        <v>46253</v>
+      </c>
       <c r="S4" t="s">
         <v>150</v>
       </c>
@@ -1208,10 +1412,13 @@
         <v>46232</v>
       </c>
       <c r="Q5" t="s">
-        <v>150</v>
+        <v>149</v>
+      </c>
+      <c r="R5">
+        <v>46253</v>
       </c>
       <c r="S5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="T5" t="s">
         <v>46</v>
@@ -1269,6 +1476,9 @@
       <c r="Q6" t="s">
         <v>150</v>
       </c>
+      <c r="R6">
+        <v>46246</v>
+      </c>
       <c r="S6" t="s">
         <v>150</v>
       </c>
@@ -1328,6 +1538,9 @@
       <c r="Q7" t="s">
         <v>150</v>
       </c>
+      <c r="R7">
+        <v>46246</v>
+      </c>
       <c r="S7" t="s">
         <v>150</v>
       </c>
@@ -1381,6 +1594,9 @@
       <c r="Q8" t="s">
         <v>150</v>
       </c>
+      <c r="R8">
+        <v>46253</v>
+      </c>
       <c r="S8" t="s">
         <v>150</v>
       </c>
@@ -1490,7 +1706,7 @@
       <c r="S10" t="s">
         <v>149</v>
       </c>
-      <c r="T10" s="2" t="s">
+      <c r="T10" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1538,12 +1754,12 @@
         <v>150</v>
       </c>
       <c r="Q11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="S11" t="s">
         <v>150</v>
       </c>
-      <c r="T11" s="3" t="s">
+      <c r="T11" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1594,15 +1810,18 @@
         <v>150</v>
       </c>
       <c r="P12">
-        <v>46247</v>
+        <v>46252</v>
       </c>
       <c r="Q12" t="s">
         <v>150</v>
       </c>
+      <c r="R12">
+        <v>46245</v>
+      </c>
       <c r="S12" t="s">
         <v>150</v>
       </c>
-      <c r="T12" s="2" t="s">
+      <c r="T12" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1836,7 +2055,10 @@
         <v>46233</v>
       </c>
       <c r="Q16" t="s">
-        <v>150</v>
+        <v>149</v>
+      </c>
+      <c r="R16">
+        <v>46251</v>
       </c>
       <c r="S16" t="s">
         <v>150</v>
@@ -1886,16 +2108,16 @@
         <v>130</v>
       </c>
       <c r="N17">
-        <v>46233</v>
+        <v>46241</v>
       </c>
       <c r="O17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P17">
-        <v>46233</v>
+        <v>46241</v>
       </c>
       <c r="Q17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="S17" t="s">
         <v>149</v>
@@ -1964,7 +2186,7 @@
       <c r="B19" t="s">
         <v>139</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19">
         <v>46266</v>
       </c>
       <c r="D19" t="s">
@@ -2003,11 +2225,764 @@
       <c r="Q19" t="s">
         <v>150</v>
       </c>
+      <c r="R19">
+        <v>46248</v>
+      </c>
       <c r="S19" t="s">
         <v>150</v>
       </c>
       <c r="T19" t="s">
         <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>7005</v>
+      </c>
+      <c r="B20" t="s">
+        <v>153</v>
+      </c>
+      <c r="C20">
+        <v>46266</v>
+      </c>
+      <c r="D20" t="s">
+        <v>154</v>
+      </c>
+      <c r="E20" t="s">
+        <v>155</v>
+      </c>
+      <c r="F20" t="s">
+        <v>156</v>
+      </c>
+      <c r="G20" t="s">
+        <v>157</v>
+      </c>
+      <c r="H20" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" t="s">
+        <v>158</v>
+      </c>
+      <c r="J20" t="s">
+        <v>159</v>
+      </c>
+      <c r="K20" t="s">
+        <v>160</v>
+      </c>
+      <c r="L20" t="s">
+        <v>26</v>
+      </c>
+      <c r="M20" t="s">
+        <v>161</v>
+      </c>
+      <c r="O20" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>150</v>
+      </c>
+      <c r="S20" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>7006</v>
+      </c>
+      <c r="B21" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21">
+        <v>46266</v>
+      </c>
+      <c r="D21" t="s">
+        <v>154</v>
+      </c>
+      <c r="E21" t="s">
+        <v>155</v>
+      </c>
+      <c r="F21" t="s">
+        <v>156</v>
+      </c>
+      <c r="G21" t="s">
+        <v>157</v>
+      </c>
+      <c r="H21" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" t="s">
+        <v>163</v>
+      </c>
+      <c r="J21" t="s">
+        <v>164</v>
+      </c>
+      <c r="K21" t="s">
+        <v>165</v>
+      </c>
+      <c r="L21" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" t="s">
+        <v>166</v>
+      </c>
+      <c r="O21" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>150</v>
+      </c>
+      <c r="S21" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>7007</v>
+      </c>
+      <c r="B22" t="s">
+        <v>167</v>
+      </c>
+      <c r="C22">
+        <v>46266</v>
+      </c>
+      <c r="D22" t="s">
+        <v>168</v>
+      </c>
+      <c r="E22" t="s">
+        <v>169</v>
+      </c>
+      <c r="F22" t="s">
+        <v>170</v>
+      </c>
+      <c r="G22" t="s">
+        <v>157</v>
+      </c>
+      <c r="H22" t="s">
+        <v>87</v>
+      </c>
+      <c r="I22" t="s">
+        <v>171</v>
+      </c>
+      <c r="J22" t="s">
+        <v>172</v>
+      </c>
+      <c r="K22" t="s">
+        <v>173</v>
+      </c>
+      <c r="L22" t="s">
+        <v>55</v>
+      </c>
+      <c r="M22" t="s">
+        <v>174</v>
+      </c>
+      <c r="O22" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>150</v>
+      </c>
+      <c r="S22" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>7012</v>
+      </c>
+      <c r="B23" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23">
+        <v>46235</v>
+      </c>
+      <c r="D23" t="s">
+        <v>176</v>
+      </c>
+      <c r="E23" t="s">
+        <v>177</v>
+      </c>
+      <c r="F23" t="s">
+        <v>178</v>
+      </c>
+      <c r="G23" t="s">
+        <v>157</v>
+      </c>
+      <c r="H23" t="s">
+        <v>96</v>
+      </c>
+      <c r="I23" t="s">
+        <v>179</v>
+      </c>
+      <c r="J23" t="s">
+        <v>180</v>
+      </c>
+      <c r="K23" t="s">
+        <v>181</v>
+      </c>
+      <c r="L23" t="s">
+        <v>55</v>
+      </c>
+      <c r="M23" t="s">
+        <v>182</v>
+      </c>
+      <c r="O23" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>150</v>
+      </c>
+      <c r="S23" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>7013</v>
+      </c>
+      <c r="B24" t="s">
+        <v>183</v>
+      </c>
+      <c r="C24">
+        <v>46235</v>
+      </c>
+      <c r="D24" t="s">
+        <v>176</v>
+      </c>
+      <c r="E24" t="s">
+        <v>177</v>
+      </c>
+      <c r="F24" t="s">
+        <v>178</v>
+      </c>
+      <c r="G24" t="s">
+        <v>157</v>
+      </c>
+      <c r="H24" t="s">
+        <v>96</v>
+      </c>
+      <c r="I24" t="s">
+        <v>184</v>
+      </c>
+      <c r="J24" t="s">
+        <v>180</v>
+      </c>
+      <c r="K24" t="s">
+        <v>181</v>
+      </c>
+      <c r="L24" t="s">
+        <v>55</v>
+      </c>
+      <c r="M24" t="s">
+        <v>185</v>
+      </c>
+      <c r="O24" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>150</v>
+      </c>
+      <c r="S24" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>7014</v>
+      </c>
+      <c r="B25" t="s">
+        <v>186</v>
+      </c>
+      <c r="C25">
+        <v>46235</v>
+      </c>
+      <c r="D25" t="s">
+        <v>176</v>
+      </c>
+      <c r="E25" t="s">
+        <v>177</v>
+      </c>
+      <c r="F25" t="s">
+        <v>178</v>
+      </c>
+      <c r="G25" t="s">
+        <v>157</v>
+      </c>
+      <c r="H25" t="s">
+        <v>87</v>
+      </c>
+      <c r="I25" t="s">
+        <v>187</v>
+      </c>
+      <c r="J25" t="s">
+        <v>188</v>
+      </c>
+      <c r="K25" t="s">
+        <v>189</v>
+      </c>
+      <c r="L25" t="s">
+        <v>190</v>
+      </c>
+      <c r="M25" t="s">
+        <v>191</v>
+      </c>
+      <c r="O25" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>150</v>
+      </c>
+      <c r="S25" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>7015</v>
+      </c>
+      <c r="B26" t="s">
+        <v>192</v>
+      </c>
+      <c r="C26">
+        <v>46235</v>
+      </c>
+      <c r="D26" t="s">
+        <v>176</v>
+      </c>
+      <c r="E26" t="s">
+        <v>177</v>
+      </c>
+      <c r="F26" t="s">
+        <v>178</v>
+      </c>
+      <c r="G26" t="s">
+        <v>157</v>
+      </c>
+      <c r="H26" t="s">
+        <v>87</v>
+      </c>
+      <c r="I26" t="s">
+        <v>193</v>
+      </c>
+      <c r="J26" t="s">
+        <v>194</v>
+      </c>
+      <c r="K26" t="s">
+        <v>181</v>
+      </c>
+      <c r="L26" t="s">
+        <v>55</v>
+      </c>
+      <c r="M26" t="s">
+        <v>220</v>
+      </c>
+      <c r="O26" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>150</v>
+      </c>
+      <c r="S26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>7016</v>
+      </c>
+      <c r="B27" t="s">
+        <v>195</v>
+      </c>
+      <c r="C27">
+        <v>46235</v>
+      </c>
+      <c r="D27" t="s">
+        <v>176</v>
+      </c>
+      <c r="E27" t="s">
+        <v>196</v>
+      </c>
+      <c r="F27" t="s">
+        <v>197</v>
+      </c>
+      <c r="G27" t="s">
+        <v>157</v>
+      </c>
+      <c r="H27" t="s">
+        <v>87</v>
+      </c>
+      <c r="I27" t="s">
+        <v>198</v>
+      </c>
+      <c r="J27" t="s">
+        <v>188</v>
+      </c>
+      <c r="K27" t="s">
+        <v>199</v>
+      </c>
+      <c r="L27" t="s">
+        <v>190</v>
+      </c>
+      <c r="M27" t="s">
+        <v>200</v>
+      </c>
+      <c r="O27" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>150</v>
+      </c>
+      <c r="S27" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>7017</v>
+      </c>
+      <c r="B28" t="s">
+        <v>201</v>
+      </c>
+      <c r="C28">
+        <v>46235</v>
+      </c>
+      <c r="D28" t="s">
+        <v>176</v>
+      </c>
+      <c r="E28" t="s">
+        <v>177</v>
+      </c>
+      <c r="F28" t="s">
+        <v>178</v>
+      </c>
+      <c r="G28" t="s">
+        <v>157</v>
+      </c>
+      <c r="H28" t="s">
+        <v>87</v>
+      </c>
+      <c r="I28" t="s">
+        <v>187</v>
+      </c>
+      <c r="J28" t="s">
+        <v>180</v>
+      </c>
+      <c r="K28" t="s">
+        <v>181</v>
+      </c>
+      <c r="L28" t="s">
+        <v>55</v>
+      </c>
+      <c r="M28" t="s">
+        <v>200</v>
+      </c>
+      <c r="O28" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>150</v>
+      </c>
+      <c r="S28" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>7018</v>
+      </c>
+      <c r="B29" t="s">
+        <v>202</v>
+      </c>
+      <c r="C29">
+        <v>46235</v>
+      </c>
+      <c r="D29" t="s">
+        <v>176</v>
+      </c>
+      <c r="E29" t="s">
+        <v>196</v>
+      </c>
+      <c r="F29" t="s">
+        <v>197</v>
+      </c>
+      <c r="G29" t="s">
+        <v>157</v>
+      </c>
+      <c r="H29" t="s">
+        <v>87</v>
+      </c>
+      <c r="I29" t="s">
+        <v>184</v>
+      </c>
+      <c r="J29" t="s">
+        <v>180</v>
+      </c>
+      <c r="K29" t="s">
+        <v>181</v>
+      </c>
+      <c r="L29" t="s">
+        <v>55</v>
+      </c>
+      <c r="M29" t="s">
+        <v>191</v>
+      </c>
+      <c r="O29" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>150</v>
+      </c>
+      <c r="S29" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>7019</v>
+      </c>
+      <c r="B30" t="s">
+        <v>203</v>
+      </c>
+      <c r="C30">
+        <v>46235</v>
+      </c>
+      <c r="D30" t="s">
+        <v>176</v>
+      </c>
+      <c r="E30" t="s">
+        <v>177</v>
+      </c>
+      <c r="F30" t="s">
+        <v>178</v>
+      </c>
+      <c r="G30" t="s">
+        <v>157</v>
+      </c>
+      <c r="H30" t="s">
+        <v>87</v>
+      </c>
+      <c r="I30" t="s">
+        <v>187</v>
+      </c>
+      <c r="J30" t="s">
+        <v>194</v>
+      </c>
+      <c r="K30" t="s">
+        <v>181</v>
+      </c>
+      <c r="L30" t="s">
+        <v>55</v>
+      </c>
+      <c r="M30" t="s">
+        <v>191</v>
+      </c>
+      <c r="O30" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>150</v>
+      </c>
+      <c r="S30" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>7020</v>
+      </c>
+      <c r="B31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C31">
+        <v>46235</v>
+      </c>
+      <c r="D31" t="s">
+        <v>176</v>
+      </c>
+      <c r="E31" t="s">
+        <v>177</v>
+      </c>
+      <c r="F31" t="s">
+        <v>178</v>
+      </c>
+      <c r="G31" t="s">
+        <v>157</v>
+      </c>
+      <c r="H31" t="s">
+        <v>87</v>
+      </c>
+      <c r="I31" t="s">
+        <v>205</v>
+      </c>
+      <c r="J31" t="s">
+        <v>188</v>
+      </c>
+      <c r="K31" t="s">
+        <v>199</v>
+      </c>
+      <c r="L31" t="s">
+        <v>190</v>
+      </c>
+      <c r="M31" t="s">
+        <v>206</v>
+      </c>
+      <c r="O31" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>150</v>
+      </c>
+      <c r="S31" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>7021</v>
+      </c>
+      <c r="B32" t="s">
+        <v>207</v>
+      </c>
+      <c r="C32">
+        <v>46235</v>
+      </c>
+      <c r="D32" t="s">
+        <v>176</v>
+      </c>
+      <c r="E32" t="s">
+        <v>196</v>
+      </c>
+      <c r="F32" t="s">
+        <v>197</v>
+      </c>
+      <c r="G32" t="s">
+        <v>157</v>
+      </c>
+      <c r="H32" t="s">
+        <v>87</v>
+      </c>
+      <c r="I32" t="s">
+        <v>198</v>
+      </c>
+      <c r="J32" t="s">
+        <v>188</v>
+      </c>
+      <c r="K32" t="s">
+        <v>199</v>
+      </c>
+      <c r="L32" t="s">
+        <v>190</v>
+      </c>
+      <c r="M32" t="s">
+        <v>206</v>
+      </c>
+      <c r="O32" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>150</v>
+      </c>
+      <c r="S32" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>6992</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C33" s="2">
+        <v>46266</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="O33" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>150</v>
+      </c>
+      <c r="S33" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>6993</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C34" s="1">
+        <v>46266</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="L34" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="M34" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="O34" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>150</v>
+      </c>
+      <c r="S34" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza base de clientes: datas de implantação e dados da 3M
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/base/base implantação.xlsx
+++ b/data/base/base implantação.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgcontecnica1-my.sharepoint.com/personal/warruda_mgcontecnica_com_br/Documents/Documentos/python/Portal-implantacao-tmp/data/base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="279" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6CD88D2-17A5-4C6C-8E30-82310FFEC7E1}"/>
+  <xr:revisionPtr revIDLastSave="346" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{659E3508-6A00-45D5-A7B9-691998C0B6CE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-1260" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="227">
   <si>
     <t>ID</t>
   </si>
@@ -683,13 +683,32 @@
   </si>
   <si>
     <t>E&amp;amp;G MARTINS PARTICIPACOES LTDA;EDUARDO DE JESUS MARTINS; AA&amp;amp;MARTINS PARTICIPACOES LTDA;ADRIANO AUGUSTO MARTINS; B&amp;amp;SOLAR PARTICIPACOES LTDA;MARCOS MARQUES MARTINS;</t>
+  </si>
+  <si>
+    <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRASIL DISTRIBUIDORA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUA DOS JUNQUILHOS, Num.: 153 Comple.: LOTE 26 - QUADRA 08 - SALA 01, Bairro: PARQUE OESTE INDUSTRIAL /
+ </t>
+  </si>
+  <si>
+    <t>brasildistribuidoradepecas@gmail.com;</t>
+  </si>
+  <si>
+    <t>(62) 8180-4195 /</t>
+  </si>
+  <si>
+    <t>CLEY MARCOS FIDELIS;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -702,6 +721,17 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -729,16 +759,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="1">
@@ -758,9 +795,13 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:T34">
-  <autoFilter ref="A1:T34" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:T35">
+  <autoFilter ref="A1:T35" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T19">
     <sortCondition ref="D1:D19"/>
   </sortState>
@@ -1107,29 +1148,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T34"/>
+  <dimension ref="A1:T35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="115.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="37.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="120.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="45.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="43.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="64.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="192" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="27" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
@@ -1337,7 +1378,7 @@
       <c r="I4" t="s">
         <v>42</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="4" t="s">
         <v>43</v>
       </c>
       <c r="K4" t="s">
@@ -1644,11 +1685,20 @@
       <c r="M9" t="s">
         <v>75</v>
       </c>
+      <c r="N9">
+        <v>46255</v>
+      </c>
       <c r="O9" t="s">
         <v>150</v>
       </c>
+      <c r="P9">
+        <v>46255</v>
+      </c>
       <c r="Q9" t="s">
         <v>150</v>
+      </c>
+      <c r="R9">
+        <v>46191</v>
       </c>
       <c r="S9" t="s">
         <v>149</v>
@@ -1697,11 +1747,20 @@
       <c r="M10" t="s">
         <v>81</v>
       </c>
+      <c r="N10">
+        <v>46255</v>
+      </c>
       <c r="O10" t="s">
         <v>150</v>
       </c>
+      <c r="P10">
+        <v>46255</v>
+      </c>
       <c r="Q10" t="s">
         <v>150</v>
+      </c>
+      <c r="R10">
+        <v>46191</v>
       </c>
       <c r="S10" t="s">
         <v>149</v>
@@ -1835,7 +1894,7 @@
       <c r="C13">
         <v>46266</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="5" t="s">
         <v>102</v>
       </c>
       <c r="E13" t="s">
@@ -2166,11 +2225,20 @@
       <c r="M18" t="s">
         <v>137</v>
       </c>
+      <c r="N18">
+        <v>46205</v>
+      </c>
       <c r="O18" t="s">
         <v>149</v>
       </c>
+      <c r="P18">
+        <v>46205</v>
+      </c>
       <c r="Q18" t="s">
         <v>149</v>
+      </c>
+      <c r="R18">
+        <v>46216</v>
       </c>
       <c r="S18" t="s">
         <v>149</v>
@@ -2437,7 +2505,7 @@
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>7013</v>
+        <v>7012</v>
       </c>
       <c r="B24" t="s">
         <v>183</v>
@@ -2931,6 +2999,9 @@
       <c r="Q33" t="s">
         <v>150</v>
       </c>
+      <c r="R33">
+        <v>46247</v>
+      </c>
       <c r="S33" t="s">
         <v>150</v>
       </c>
@@ -2981,14 +3052,80 @@
       <c r="Q34" t="s">
         <v>150</v>
       </c>
+      <c r="R34">
+        <v>46247</v>
+      </c>
       <c r="S34" t="s">
         <v>150</v>
       </c>
     </row>
+    <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>6945</v>
+      </c>
+      <c r="B35" t="s">
+        <v>221</v>
+      </c>
+      <c r="C35" s="1">
+        <v>46174</v>
+      </c>
+      <c r="D35" t="s">
+        <v>222</v>
+      </c>
+      <c r="E35" t="s">
+        <v>155</v>
+      </c>
+      <c r="F35" t="s">
+        <v>156</v>
+      </c>
+      <c r="G35" t="s">
+        <v>157</v>
+      </c>
+      <c r="H35" t="s">
+        <v>22</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="K35" t="s">
+        <v>225</v>
+      </c>
+      <c r="L35" t="s">
+        <v>26</v>
+      </c>
+      <c r="M35" t="s">
+        <v>226</v>
+      </c>
+      <c r="N35">
+        <v>46219</v>
+      </c>
+      <c r="O35" t="s">
+        <v>150</v>
+      </c>
+      <c r="P35">
+        <v>46219</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>150</v>
+      </c>
+      <c r="R35">
+        <v>46217</v>
+      </c>
+      <c r="S35" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J4" r:id="rId1" xr:uid="{0FBB74B0-7BDF-4CCB-902E-06F540839053}"/>
+    <hyperlink ref="J35" r:id="rId2" xr:uid="{66BBE0A7-BDDD-4208-88F5-EC986E31CB14}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza planilha de implantação (sync automático)
</commit_message>
<xml_diff>
--- a/data/base/base implantação.xlsx
+++ b/data/base/base implantação.xlsx
@@ -1,21 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgcontecnica1-my.sharepoint.com/personal/warruda_mgcontecnica_com_br/Documents/Documentos/python/Portal-implantacao-tmp/data/base/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="357" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F4ABBC1-7B23-4103-8804-46AA31A8F007}"/>
+  <xr:revisionPtr revIDLastSave="391" documentId="11_4F56B3A8CB9C0E20059044E3BFE40D0DED129F61" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFDA0571-C6BB-4559-BB8F-B18A0B54658E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -64,12 +80,21 @@
     <t>Implantação CTB</t>
   </si>
   <si>
+    <t>Implantação CTB - Realizada</t>
+  </si>
+  <si>
     <t>Implantação EF</t>
   </si>
   <si>
+    <t>Implantação EF - Realizada</t>
+  </si>
+  <si>
     <t>Implantação DP</t>
   </si>
   <si>
+    <t>Implantação DP - Realizada</t>
+  </si>
+  <si>
     <t>GrupoID</t>
   </si>
   <si>
@@ -106,6 +131,9 @@
     <t>RAFAELA YUMI TUKAMOTO;</t>
   </si>
   <si>
+    <t>Não</t>
+  </si>
+  <si>
     <t>atria-cenografia</t>
   </si>
   <si>
@@ -160,6 +188,9 @@
     <t>JACINTO DE OLIVEIRA NETO;CÁRITAS NEIVA VIEIRA FRANÇA;</t>
   </si>
   <si>
+    <t>Sim</t>
+  </si>
+  <si>
     <t>film-facil</t>
   </si>
   <si>
@@ -298,6 +329,9 @@
     <t>JOEL CHERUBIM DE BARROS;</t>
   </si>
   <si>
+    <t>lagoa-bonita</t>
+  </si>
+  <si>
     <t>SUPER DIJAN COMERCIAL LTDA</t>
   </si>
   <si>
@@ -325,6 +359,9 @@
     <t>JANDUI RODRIGUES DE MIRANDA; FELIPE DIJAN SANTOS DE MIRANDA;</t>
   </si>
   <si>
+    <t>mercado-dijan</t>
+  </si>
+  <si>
     <t>F. MARQUES DE SA LTDA</t>
   </si>
   <si>
@@ -460,27 +497,6 @@
     <t>trizga</t>
   </si>
   <si>
-    <t>Implantação CTB - Realizada</t>
-  </si>
-  <si>
-    <t>Implantação EF - Realizada</t>
-  </si>
-  <si>
-    <t>Implantação DP - Realizada</t>
-  </si>
-  <si>
-    <t>Sim</t>
-  </si>
-  <si>
-    <t>Não</t>
-  </si>
-  <si>
-    <t>mercado-dijan</t>
-  </si>
-  <si>
-    <t>lagoa-bonita</t>
-  </si>
-  <si>
     <t>INDEP INDUSTRIA E COMERCIO DE PLASTICOS LTDA</t>
   </si>
   <si>
@@ -607,6 +623,9 @@
     <t>contabil@supermercados3m.com.br;</t>
   </si>
   <si>
+    <t>E&amp;amp;G MARTINS PARTICIPACOES LTDA;EDUARDO DE JESUS MARTINS; AA&amp;amp;MARTINS PARTICIPACOES LTDA;ADRIANO AUGUSTO MARTINS; B&amp;amp;SOLAR PARTICIPACOES LTDA;MARCOS MARQUES MARTINS;</t>
+  </si>
+  <si>
     <t>E&amp;G MARTINS PARTICIPAÇÕES LTDA</t>
   </si>
   <si>
@@ -655,21 +674,21 @@
     <t>Ricardo Ferreira;</t>
   </si>
   <si>
+    <t xml:space="preserve">RUA JERÔNIMO VILELA, Num.: 271 Comple.: QUADRA 27 LOTE 13, Bairro: VILA SOFIA / </t>
+  </si>
+  <si>
+    <t>venanciopardal@hotmail.com;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">64 996444975 / </t>
+  </si>
+  <si>
+    <t>ALDENIR VENANCIO DE OLIVEIRA;</t>
+  </si>
+  <si>
     <t>GOMES SERVIÇOS - LTDA</t>
   </si>
   <si>
-    <t xml:space="preserve">RUA JERÔNIMO VILELA, Num.: 271 Comple.: QUADRA 27 LOTE 13, Bairro: VILA SOFIA / </t>
-  </si>
-  <si>
-    <t>venanciopardal@hotmail.com;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">64 996444975 / </t>
-  </si>
-  <si>
-    <t>ALDENIR VENANCIO DE OLIVEIRA;</t>
-  </si>
-  <si>
     <t xml:space="preserve">RUA MINAS GERAIS, Num.: 698 Comple.: QUADRA 48 - LOTE 10A - SALA 01, Bairro: VILA SANTA MARIA / </t>
   </si>
   <si>
@@ -680,9 +699,6 @@
   </si>
   <si>
     <t>ARMANDO GOMES DE ASSIS;</t>
-  </si>
-  <si>
-    <t>E&amp;amp;G MARTINS PARTICIPACOES LTDA;EDUARDO DE JESUS MARTINS; AA&amp;amp;MARTINS PARTICIPACOES LTDA;ADRIANO AUGUSTO MARTINS; B&amp;amp;SOLAR PARTICIPACOES LTDA;MARCOS MARQUES MARTINS;</t>
   </si>
   <si>
     <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
@@ -708,7 +724,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -763,7 +779,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -773,12 +789,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
@@ -795,10 +821,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:T35">
   <autoFilter ref="A1:T35" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -808,7 +830,7 @@
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" totalsRowFunction="average"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="RazaoSocial" totalsRowFunction="average"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ContratoMG" totalsRowFunction="average" dataDxfId="0"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="ContratoMG" totalsRowFunction="average" dataDxfId="3"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Grupo" totalsRowFunction="average"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Gerente" totalsRowFunction="average"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Secretaria" totalsRowFunction="average"/>
@@ -819,11 +841,11 @@
     <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Telefone" totalsRowFunction="average"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Segmento" totalsRowFunction="average"/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Socio" totalsRowFunction="average"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Implantação CTB"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Implantação CTB" dataDxfId="2"/>
     <tableColumn id="7" xr3:uid="{0AFAB906-C921-447F-AE27-262AE6DF88B4}" name="Implantação CTB - Realizada"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Implantação EF"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Implantação EF" dataDxfId="1"/>
     <tableColumn id="8" xr3:uid="{5B2D038A-745A-4A1C-8CCD-0A7265A0AA57}" name="Implantação EF - Realizada"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Implantação DP"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Implantação DP" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{4EC4A72A-B6C2-47C3-A66B-DB898C2CE30E}" name="Implantação DP - Realizada"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="GrupoID"/>
   </tableColumns>
@@ -1149,31 +1171,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="72.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="120.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="45.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="43.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.140625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="45.42578125" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="43.28515625" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="192" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="192" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="18" style="7" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.7109375" style="7" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="27" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.7109375" style="7" customWidth="1"/>
     <col min="19" max="19" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1213,1097 +1236,1097 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>146</v>
-      </c>
-      <c r="P1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="Q1" t="s">
-        <v>147</v>
-      </c>
-      <c r="R1" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="R1" s="7" t="s">
+        <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>148</v>
+        <v>18</v>
       </c>
       <c r="T1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
       <c r="A2">
         <v>6989</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>46220</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="J2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="K2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="O2" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q2" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S2" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20">
       <c r="A3">
         <v>6812</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C3">
         <v>46266</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="J3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="K3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>37</v>
-      </c>
-      <c r="N3">
+        <v>41</v>
+      </c>
+      <c r="N3" s="7">
         <v>46260</v>
       </c>
       <c r="O3" t="s">
-        <v>150</v>
-      </c>
-      <c r="P3">
+        <v>31</v>
+      </c>
+      <c r="P3" s="7">
         <v>46260</v>
       </c>
       <c r="Q3" t="s">
-        <v>150</v>
-      </c>
-      <c r="R3">
+        <v>31</v>
+      </c>
+      <c r="R3" s="7">
         <v>46251</v>
       </c>
       <c r="S3" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20">
       <c r="A4">
         <v>6976</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C4">
         <v>46235</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M4" t="s">
-        <v>45</v>
-      </c>
-      <c r="N4">
+        <v>49</v>
+      </c>
+      <c r="N4" s="7">
         <v>46232</v>
       </c>
       <c r="O4" t="s">
-        <v>150</v>
-      </c>
-      <c r="P4">
+        <v>31</v>
+      </c>
+      <c r="P4" s="7">
         <v>46232</v>
       </c>
       <c r="Q4" t="s">
-        <v>149</v>
-      </c>
-      <c r="R4">
+        <v>50</v>
+      </c>
+      <c r="R4" s="7">
         <v>46253</v>
       </c>
       <c r="S4" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20">
       <c r="A5">
         <v>6977</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C5">
         <v>46235</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="L5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M5" t="s">
-        <v>48</v>
-      </c>
-      <c r="N5">
+        <v>53</v>
+      </c>
+      <c r="N5" s="7">
         <v>46232</v>
       </c>
       <c r="O5" t="s">
-        <v>150</v>
-      </c>
-      <c r="P5">
+        <v>31</v>
+      </c>
+      <c r="P5" s="7">
         <v>46232</v>
       </c>
       <c r="Q5" t="s">
-        <v>149</v>
-      </c>
-      <c r="R5">
+        <v>50</v>
+      </c>
+      <c r="R5" s="7">
         <v>46253</v>
       </c>
       <c r="S5" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20">
       <c r="A6">
         <v>6966</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C6">
         <v>46235</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I6" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="J6" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="K6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="L6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M6" t="s">
-        <v>56</v>
-      </c>
-      <c r="N6">
+        <v>61</v>
+      </c>
+      <c r="N6" s="7">
         <v>46245</v>
       </c>
       <c r="O6" t="s">
-        <v>150</v>
-      </c>
-      <c r="P6">
+        <v>31</v>
+      </c>
+      <c r="P6" s="7">
         <v>46245</v>
       </c>
       <c r="Q6" t="s">
-        <v>150</v>
-      </c>
-      <c r="R6">
+        <v>31</v>
+      </c>
+      <c r="R6" s="7">
         <v>46246</v>
       </c>
       <c r="S6" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20">
       <c r="A7">
         <v>6967</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>46235</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="J7" t="s">
+        <v>65</v>
+      </c>
+      <c r="K7" t="s">
+        <v>66</v>
+      </c>
+      <c r="L7" t="s">
         <v>60</v>
       </c>
-      <c r="K7" t="s">
-        <v>61</v>
-      </c>
-      <c r="L7" t="s">
-        <v>55</v>
-      </c>
       <c r="M7" t="s">
+        <v>67</v>
+      </c>
+      <c r="N7" s="7">
+        <v>46245</v>
+      </c>
+      <c r="O7" t="s">
+        <v>31</v>
+      </c>
+      <c r="P7" s="7">
+        <v>46245</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" s="7">
+        <v>46246</v>
+      </c>
+      <c r="S7" t="s">
+        <v>31</v>
+      </c>
+      <c r="T7" t="s">
         <v>62</v>
       </c>
-      <c r="N7">
-        <v>46245</v>
-      </c>
-      <c r="O7" t="s">
-        <v>150</v>
-      </c>
-      <c r="P7">
-        <v>46245</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>150</v>
-      </c>
-      <c r="R7">
-        <v>46246</v>
-      </c>
-      <c r="S7" t="s">
-        <v>150</v>
-      </c>
-      <c r="T7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:20">
       <c r="A8">
         <v>6978</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C8">
         <v>46266</v>
       </c>
       <c r="D8" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="J8" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="K8" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="O8" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q8" t="s">
-        <v>150</v>
-      </c>
-      <c r="R8">
+        <v>31</v>
+      </c>
+      <c r="R8" s="7">
         <v>46253</v>
       </c>
       <c r="S8" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T8" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20">
       <c r="A9">
         <v>6923</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C9">
         <v>46204</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G9" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="K9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="L9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M9" t="s">
-        <v>75</v>
-      </c>
-      <c r="N9">
+        <v>80</v>
+      </c>
+      <c r="N9" s="7">
         <v>46255</v>
       </c>
       <c r="O9" t="s">
-        <v>150</v>
-      </c>
-      <c r="P9">
+        <v>31</v>
+      </c>
+      <c r="P9" s="7">
         <v>46255</v>
       </c>
       <c r="Q9" t="s">
-        <v>150</v>
-      </c>
-      <c r="R9">
+        <v>31</v>
+      </c>
+      <c r="R9" s="7">
         <v>46191</v>
       </c>
       <c r="S9" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="T9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20">
       <c r="A10">
         <v>6924</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C10">
         <v>46204</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E10" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I10" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="J10" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="K10" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="L10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M10" t="s">
+        <v>86</v>
+      </c>
+      <c r="N10" s="7">
+        <v>46255</v>
+      </c>
+      <c r="O10" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="7">
+        <v>46255</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>31</v>
+      </c>
+      <c r="R10" s="7">
+        <v>46191</v>
+      </c>
+      <c r="S10" t="s">
+        <v>50</v>
+      </c>
+      <c r="T10" t="s">
         <v>81</v>
       </c>
-      <c r="N10">
-        <v>46255</v>
-      </c>
-      <c r="O10" t="s">
-        <v>150</v>
-      </c>
-      <c r="P10">
-        <v>46255</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>150</v>
-      </c>
-      <c r="R10">
-        <v>46191</v>
-      </c>
-      <c r="S10" t="s">
-        <v>149</v>
-      </c>
-      <c r="T10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:20">
       <c r="A11">
         <v>6850</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C11">
         <v>46204</v>
       </c>
       <c r="D11" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E11" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G11" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="H11" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I11" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="J11" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="K11" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="L11" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M11" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="O11" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q11" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="S11" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T11" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20">
       <c r="A12">
         <v>6964</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C12">
         <v>46235</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E12" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F12" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J12" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="K12" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L12" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M12" t="s">
-        <v>100</v>
-      </c>
-      <c r="N12">
+        <v>106</v>
+      </c>
+      <c r="N12" s="7">
         <v>46247</v>
       </c>
       <c r="O12" t="s">
-        <v>150</v>
-      </c>
-      <c r="P12">
+        <v>31</v>
+      </c>
+      <c r="P12" s="7">
         <v>46252</v>
       </c>
       <c r="Q12" t="s">
-        <v>150</v>
-      </c>
-      <c r="R12">
+        <v>31</v>
+      </c>
+      <c r="R12" s="7">
         <v>46245</v>
       </c>
       <c r="S12" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T12" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20">
       <c r="A13">
         <v>6947</v>
       </c>
       <c r="B13" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="C13">
         <v>46266</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" t="s">
+        <v>45</v>
+      </c>
+      <c r="H13" t="s">
         <v>102</v>
       </c>
-      <c r="E13" t="s">
-        <v>31</v>
-      </c>
-      <c r="F13" t="s">
-        <v>32</v>
-      </c>
-      <c r="G13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H13" t="s">
-        <v>96</v>
-      </c>
       <c r="I13" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="J13" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="K13" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="L13" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M13" t="s">
-        <v>106</v>
-      </c>
-      <c r="N13">
+        <v>113</v>
+      </c>
+      <c r="N13" s="7">
         <v>46259</v>
       </c>
       <c r="O13" t="s">
-        <v>150</v>
-      </c>
-      <c r="P13">
+        <v>31</v>
+      </c>
+      <c r="P13" s="7">
         <v>46259</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="R13">
+        <v>31</v>
+      </c>
+      <c r="R13" s="7">
         <v>46245</v>
       </c>
       <c r="S13" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T13" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20">
       <c r="A14">
         <v>6962</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C14">
         <v>46174</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="E14" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H14" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I14" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="J14" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="K14" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="L14" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M14" t="s">
-        <v>113</v>
-      </c>
-      <c r="N14">
+        <v>120</v>
+      </c>
+      <c r="N14" s="7">
         <v>46232</v>
       </c>
       <c r="O14" t="s">
-        <v>149</v>
-      </c>
-      <c r="P14">
+        <v>50</v>
+      </c>
+      <c r="P14" s="7">
         <v>46232</v>
       </c>
       <c r="Q14" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S14" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="T14" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20">
       <c r="A15">
         <v>6963</v>
       </c>
       <c r="B15" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="C15">
         <v>46174</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H15" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I15" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="J15" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="K15" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="L15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M15" t="s">
-        <v>113</v>
-      </c>
-      <c r="N15">
+        <v>120</v>
+      </c>
+      <c r="N15" s="7">
         <v>46232</v>
       </c>
       <c r="O15" t="s">
-        <v>149</v>
-      </c>
-      <c r="P15">
+        <v>50</v>
+      </c>
+      <c r="P15" s="7">
         <v>46232</v>
       </c>
       <c r="Q15" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S15" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="T15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20">
       <c r="A16">
         <v>6981</v>
       </c>
       <c r="B16" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C16">
         <v>46235</v>
       </c>
       <c r="D16" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G16" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H16" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I16" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="J16" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="K16" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="L16" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M16" t="s">
-        <v>123</v>
-      </c>
-      <c r="N16">
+        <v>130</v>
+      </c>
+      <c r="N16" s="7">
         <v>46233</v>
       </c>
       <c r="O16" t="s">
-        <v>150</v>
-      </c>
-      <c r="P16">
+        <v>31</v>
+      </c>
+      <c r="P16" s="7">
         <v>46233</v>
       </c>
       <c r="Q16" t="s">
-        <v>149</v>
-      </c>
-      <c r="R16">
+        <v>50</v>
+      </c>
+      <c r="R16" s="7">
         <v>46251</v>
       </c>
       <c r="S16" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T16" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20">
       <c r="A17">
         <v>6974</v>
       </c>
       <c r="B17" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="C17">
         <v>46204</v>
       </c>
       <c r="D17" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="E17" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G17" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H17" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I17" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="J17" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="K17" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="L17" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M17" t="s">
-        <v>130</v>
-      </c>
-      <c r="N17">
+        <v>137</v>
+      </c>
+      <c r="N17" s="7">
         <v>46241</v>
       </c>
       <c r="O17" t="s">
-        <v>149</v>
-      </c>
-      <c r="P17">
+        <v>50</v>
+      </c>
+      <c r="P17" s="7">
         <v>46241</v>
       </c>
       <c r="Q17" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="S17" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="T17" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20">
       <c r="A18">
         <v>6949</v>
       </c>
       <c r="B18" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C18">
         <v>46204</v>
       </c>
       <c r="D18" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E18" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="F18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H18" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I18" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="J18" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="K18" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="L18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M18" t="s">
-        <v>137</v>
-      </c>
-      <c r="N18">
+        <v>144</v>
+      </c>
+      <c r="N18" s="7">
         <v>46205</v>
       </c>
       <c r="O18" t="s">
-        <v>149</v>
-      </c>
-      <c r="P18">
+        <v>50</v>
+      </c>
+      <c r="P18" s="7">
         <v>46205</v>
       </c>
       <c r="Q18" t="s">
-        <v>149</v>
-      </c>
-      <c r="R18">
+        <v>50</v>
+      </c>
+      <c r="R18" s="7">
         <v>46216</v>
       </c>
       <c r="S18" t="s">
-        <v>149</v>
+        <v>50</v>
       </c>
       <c r="T18" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20">
       <c r="A19">
         <v>6995</v>
       </c>
       <c r="B19" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C19">
         <v>46266</v>
       </c>
       <c r="D19" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F19" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H19" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I19" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="J19" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="K19" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="L19" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M19" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="O19" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q19" t="s">
-        <v>150</v>
-      </c>
-      <c r="R19">
+        <v>31</v>
+      </c>
+      <c r="R19" s="7">
         <v>46248</v>
       </c>
       <c r="S19" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="T19" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20">
       <c r="A20">
         <v>7005</v>
       </c>
@@ -2326,7 +2349,7 @@
         <v>157</v>
       </c>
       <c r="H20" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I20" t="s">
         <v>158</v>
@@ -2338,22 +2361,22 @@
         <v>160</v>
       </c>
       <c r="L20" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M20" t="s">
         <v>161</v>
       </c>
       <c r="O20" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q20" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S20" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20">
       <c r="A21">
         <v>7006</v>
       </c>
@@ -2376,7 +2399,7 @@
         <v>157</v>
       </c>
       <c r="H21" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I21" t="s">
         <v>163</v>
@@ -2388,22 +2411,22 @@
         <v>165</v>
       </c>
       <c r="L21" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M21" t="s">
         <v>166</v>
       </c>
       <c r="O21" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q21" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S21" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20">
       <c r="A22">
         <v>7007</v>
       </c>
@@ -2426,7 +2449,7 @@
         <v>157</v>
       </c>
       <c r="H22" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I22" t="s">
         <v>171</v>
@@ -2438,22 +2461,22 @@
         <v>173</v>
       </c>
       <c r="L22" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M22" t="s">
         <v>174</v>
       </c>
       <c r="O22" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q22" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S22" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20">
       <c r="A23">
         <v>7012</v>
       </c>
@@ -2476,7 +2499,7 @@
         <v>157</v>
       </c>
       <c r="H23" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I23" t="s">
         <v>179</v>
@@ -2488,22 +2511,22 @@
         <v>181</v>
       </c>
       <c r="L23" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M23" t="s">
         <v>182</v>
       </c>
       <c r="O23" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q23" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S23" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20">
       <c r="A24">
         <v>7012</v>
       </c>
@@ -2526,7 +2549,7 @@
         <v>157</v>
       </c>
       <c r="H24" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I24" t="s">
         <v>184</v>
@@ -2538,22 +2561,22 @@
         <v>181</v>
       </c>
       <c r="L24" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M24" t="s">
         <v>185</v>
       </c>
       <c r="O24" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q24" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S24" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20">
       <c r="A25">
         <v>7014</v>
       </c>
@@ -2576,7 +2599,7 @@
         <v>157</v>
       </c>
       <c r="H25" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I25" t="s">
         <v>187</v>
@@ -2594,16 +2617,16 @@
         <v>191</v>
       </c>
       <c r="O25" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q25" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S25" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20">
       <c r="A26">
         <v>7015</v>
       </c>
@@ -2626,7 +2649,7 @@
         <v>157</v>
       </c>
       <c r="H26" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I26" t="s">
         <v>193</v>
@@ -2638,27 +2661,27 @@
         <v>181</v>
       </c>
       <c r="L26" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M26" t="s">
-        <v>220</v>
+        <v>195</v>
       </c>
       <c r="O26" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q26" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S26" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20">
       <c r="A27">
         <v>7016</v>
       </c>
       <c r="B27" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C27">
         <v>46235</v>
@@ -2667,48 +2690,48 @@
         <v>176</v>
       </c>
       <c r="E27" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F27" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G27" t="s">
         <v>157</v>
       </c>
       <c r="H27" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I27" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J27" t="s">
         <v>188</v>
       </c>
       <c r="K27" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L27" t="s">
         <v>190</v>
       </c>
       <c r="M27" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O27" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q27" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S27" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20">
       <c r="A28">
         <v>7017</v>
       </c>
       <c r="B28" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C28">
         <v>46235</v>
@@ -2726,7 +2749,7 @@
         <v>157</v>
       </c>
       <c r="H28" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I28" t="s">
         <v>187</v>
@@ -2738,27 +2761,27 @@
         <v>181</v>
       </c>
       <c r="L28" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M28" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O28" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q28" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S28" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20">
       <c r="A29">
         <v>7018</v>
       </c>
       <c r="B29" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C29">
         <v>46235</v>
@@ -2767,16 +2790,16 @@
         <v>176</v>
       </c>
       <c r="E29" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F29" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G29" t="s">
         <v>157</v>
       </c>
       <c r="H29" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I29" t="s">
         <v>184</v>
@@ -2788,27 +2811,27 @@
         <v>181</v>
       </c>
       <c r="L29" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M29" t="s">
         <v>191</v>
       </c>
       <c r="O29" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q29" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S29" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20">
       <c r="A30">
         <v>7019</v>
       </c>
       <c r="B30" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C30">
         <v>46235</v>
@@ -2826,7 +2849,7 @@
         <v>157</v>
       </c>
       <c r="H30" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I30" t="s">
         <v>187</v>
@@ -2838,27 +2861,27 @@
         <v>181</v>
       </c>
       <c r="L30" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M30" t="s">
         <v>191</v>
       </c>
       <c r="O30" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q30" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S30" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20">
       <c r="A31">
         <v>7020</v>
       </c>
       <c r="B31" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C31">
         <v>46235</v>
@@ -2876,39 +2899,39 @@
         <v>157</v>
       </c>
       <c r="H31" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I31" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J31" t="s">
         <v>188</v>
       </c>
       <c r="K31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L31" t="s">
         <v>190</v>
       </c>
       <c r="M31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O31" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q31" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S31" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20">
       <c r="A32">
         <v>7021</v>
       </c>
       <c r="B32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C32">
         <v>46235</v>
@@ -2917,57 +2940,57 @@
         <v>176</v>
       </c>
       <c r="E32" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F32" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G32" t="s">
         <v>157</v>
       </c>
       <c r="H32" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I32" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="J32" t="s">
         <v>188</v>
       </c>
       <c r="K32" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L32" t="s">
         <v>190</v>
       </c>
       <c r="M32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O32" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q32" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="S32" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19">
       <c r="A33" s="2">
         <v>6992</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C33" s="2">
         <v>46266</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>156</v>
@@ -2976,7 +2999,7 @@
         <v>157</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>212</v>
@@ -2988,39 +3011,39 @@
         <v>214</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M33" s="2" t="s">
         <v>215</v>
       </c>
       <c r="O33" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q33" t="s">
-        <v>150</v>
-      </c>
-      <c r="R33">
+        <v>31</v>
+      </c>
+      <c r="R33" s="7">
         <v>46247</v>
       </c>
       <c r="S33" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19">
       <c r="A34" s="3">
         <v>6993</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C34" s="1">
         <v>46266</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>156</v>
@@ -3029,37 +3052,37 @@
         <v>157</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O34" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
       <c r="Q34" t="s">
-        <v>150</v>
-      </c>
-      <c r="R34">
+        <v>31</v>
+      </c>
+      <c r="R34" s="7">
         <v>46247</v>
       </c>
       <c r="S34" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="30">
       <c r="A35">
         <v>6945</v>
       </c>
@@ -3082,7 +3105,7 @@
         <v>157</v>
       </c>
       <c r="H35" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>223</v>
@@ -3094,31 +3117,54 @@
         <v>225</v>
       </c>
       <c r="L35" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="M35" t="s">
         <v>226</v>
       </c>
-      <c r="N35">
+      <c r="N35" s="7">
         <v>46219</v>
       </c>
       <c r="O35" t="s">
-        <v>150</v>
-      </c>
-      <c r="P35">
+        <v>31</v>
+      </c>
+      <c r="P35" s="7">
         <v>46219</v>
       </c>
       <c r="Q35" t="s">
-        <v>150</v>
-      </c>
-      <c r="R35">
+        <v>31</v>
+      </c>
+      <c r="R35" s="7">
         <v>46217</v>
       </c>
       <c r="S35" t="s">
-        <v>150</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="6">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="O valor digitado deve ser uma data." promptTitle="Insira uma data " prompt="Use o formato dd/mm/aaaa" sqref="P1:P1048576" xr:uid="{C38150F2-07B9-4A40-94E9-2F60486C9785}">
+      <formula1>46023</formula1>
+      <formula2>46387</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Insira uma data" error="O valor digitado deve ser uma data." promptTitle="Insira uma data" prompt="Use o formato dd/mm/aaaa" sqref="N1:N1048576" xr:uid="{E30AD5C4-327F-471C-A8FE-8847233F32A8}">
+      <formula1>46023</formula1>
+      <formula2>46387</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="O valor digitado deve ser uma data." promptTitle="Insira uma data" prompt="Use o formato dd/mm/aaaa" sqref="R1:R1048576" xr:uid="{B80591A4-C609-4DDF-A9CB-595A54330A1C}">
+      <formula1>46023</formula1>
+      <formula2>46387</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Sim ou Não" promptTitle="Sim ou Não" sqref="O1:O6 O8:O1048576" xr:uid="{AB8A33F0-C3A3-4068-930A-A486B539D982}">
+      <formula1>"Sim;Não"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Sim ou Não" promptTitle="Sim ou Não" sqref="O7 Q1:Q1048576" xr:uid="{A33B9050-2903-44EC-9C32-C551C6DD218F}">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S1:S1048576" xr:uid="{F98435C8-1E0D-420B-93AD-1750A0AD1E4D}">
+      <formula1>"Sim,Não"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="J4" r:id="rId1" xr:uid="{0FBB74B0-7BDF-4CCB-902E-06F540839053}"/>
     <hyperlink ref="J35" r:id="rId2" xr:uid="{66BBE0A7-BDDD-4208-88F5-EC986E31CB14}"/>

</xml_diff>